<commit_message>
auto: inverter data update
</commit_message>
<xml_diff>
--- a/inverter_log.xlsx
+++ b/inverter_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,6 +524,39 @@
         <v>1445</v>
       </c>
       <c r="I3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-11 16:17:35</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>220</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1445</v>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>

</xml_diff>